<commit_message>
Switch Forwardtester to a single tenure-window Monte Carlo.
All paths share Start=as-of and End=Product End with N independent GBM seeds (default 100), replacing staggered frequency starts and Simulation End Days.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Product_Input_File.xlsx
+++ b/Product_Input_File.xlsx
@@ -751,11 +751,11 @@
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>Simulation End Days</t>
+          <t>Monte Carlo Paths</t>
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>7300</v>
+        <v>100</v>
       </c>
     </row>
     <row r="20" ht="28" customHeight="1">

</xml_diff>